<commit_message>
Add original-vs-merged mapping sheet covering all 97 questions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SvhhmDmJmcdpK13xwA7pox
</commit_message>
<xml_diff>
--- a/docs/global-ar-survey-merged.xlsx
+++ b/docs/global-ar-survey-merged.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="說明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="題目與選項" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="刪減對照" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="原始vs合併對照" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="統計" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'題目與選項'!$A$1:$H$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'原始vs合併對照'!$A$1:$F$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +53,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -93,6 +109,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -501,7 +526,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>「原題號」欄標示每題對應的原 97 題;「刪減對照」分頁列出被刪減的細項及處理方式。</t>
+          <t>「原題號」欄標示每題對應的原 97 題;「原始vs合併對照」分頁逐題列出 97 題的處理方式(保留 / 簡化 / 合併 / 刪除)及差異說明。</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1230,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>B11, B12, B13</t>
+          <t>B11, B12</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -2232,7 +2257,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>D12, D13, D14</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2509,7 +2534,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>E6, E7, E8, E9</t>
+          <t>E6, E7, E8</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -3006,7 +3031,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>G4, G5, G6, F8</t>
+          <t>G5, G6, F8</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -3144,7 +3169,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>H4, H6</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -3235,7 +3260,7 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>H7, H8, H13</t>
+          <t>H7, H8</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -3417,12 +3442,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3433,305 +3461,3136 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>被刪減 / 合併的細項</t>
+          <t>區塊</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>處理方式</t>
+          <t>原題摘要</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>處理</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>新題號</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>差異說明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>A8</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>提單數、Outstanding 筆數</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>A5–A7 只保留帳單數、收款筆數、Outstanding 金額</t>
+          <t>收款作業涵蓋項目</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>選項採原題舉例,無變動</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>B5/B7</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>開立時點、開立幣別、系統</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>系統併入 B2;幣別併入 C2</t>
+          <t>進口收款作業流程</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>開放式流程說明改為「分工模式」單選;與 A3、A7 合併;流程細節改由訪談</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>B6/B8</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>進口 / 出口分開問</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>合併為 B5</t>
+          <t>出口收款作業流程</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>併入 A2,進口與出口不再分開問</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>銀行帳戶數及區分</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>刪減,建議訪談補</t>
+          <t>收款與銷帳負責單位</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>選項採原題列舉的單位</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>付款明細內容</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>併入 D2</t>
+          <t>日班與夜班分工</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>與 A6 合併為一題「分工及交接」</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>D3-1</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>比對系統清單</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>刪減</t>
+          <t>日夜班未完成案件交接及追蹤</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>併入 A4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>D12–D14</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>退款原因、時效、方式、幣別、帳戶</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>僅保留核准層級(D10)</t>
+          <t>在地與 ICBO 集中處理的分工</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>併入 A2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>E2-2</t>
+          <t>A8</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>逾期認定方式</t>
+          <t>A. 基本資料及作業範圍</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>刪減</t>
+          <t>每月提單數、帳單數、收款/銷帳筆數、Outstanding 筆數與金額</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>A5, A6, A7</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>6 個數字縮成 3 題:帳單數、收款及銷帳筆數、Outstanding 金額;刪除提單數與 Outstanding 筆數;數字改為區間</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Web / Telex Release 執行單位及系統</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>刪減,建議訪談補</t>
+          <t>應收帳款成立時點</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>第三地付款放貨</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>併入 G4</t>
+          <t>應收帳款資料來源</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>與 B3 合併</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>第三地付款幣別 / 帳戶</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>刪減</t>
+          <t>Manifest / Non-Manifest 建檔系統</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>併入 B2,兩類費用不再分開問系統</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>G7–G9</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>C/A 通知、第三地付款退款</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>刪減,退款併入 D10</t>
+          <t>發票/帳單開立層級</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>H2-2</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Non-Manifest / Local Charge 費用項目</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>刪減,建議訪談補</t>
+          <t>進口開立流程(單位、時點、方式、幣別、系統)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>5 項縮為「由誰、以何種方式開立」;刪除開立時點;幣別併入 C2;系統併入 B2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>B6</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>LFC 產製 / 檢核 / 核准 / 送檔單位</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>刪減,建議訪談補</t>
+          <t>進口帳單辨識(獨立編號 / 付款依據)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>與 B8 合併,進口與出口不再分開</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>H9</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>匯款頻率、Cut-off、換匯時點</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>FRMD 分頁已有匯款頻率,可預填</t>
+          <t>出口開立流程(單位、時點、方式、幣別、系統)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>併入 B4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>H12</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>匯款扣除項目</t>
+          <t>B. 應收帳款及帳單開立</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>刪減,FRMD 分頁已有手續費資料</t>
+          <t>出口帳單辨識</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>併入 B5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>B9</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>特殊費用的開立單位、時點、幣別、收款流程</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>B9</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>4 項縮為 1 題:流程是否與運費相同(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>應收資料可連結的資訊</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>選項同原題舉例(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>B11</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Due Date 計算方式</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>與 B12 合併</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>B12</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>授信客戶 Due Date;Manifest 與 Non-Manifest 是否相同</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>併入 B6;「兩類費用是否相同」子問題刪除</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>B13</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>帳單異動情況及是否影響 Due Date</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>只保留「是否留存異動紀錄」;刪除異動情況清單及對 Due Date 的影響</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>B14</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>異動由哪個單位執行、是否保留紀錄</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>併入 B7;刪除執行單位</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>B15</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>B. 應收帳款及帳單開立</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Payment Center 流程(使用與否、系統、傳輸、查詢)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>B8</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>4 項縮為 1 題:使用程度(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>客戶付款方式</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>付款幣別、是否須與帳單一致、兩類費用是否不同</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>3 項縮為 1 題;刪除可用幣別清單(FRMD 分頁已有幣別資料)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>匯入銀行帳戶及區分方式</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>刪除,細節建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>銀行明細取得方式</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>取得頻率及付款後多久可取得</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>只保留「付款後多久取得」;刪除取得頻率</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>銀行明細可提供欄位</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>客戶付款明細取得方式</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>客戶付款明細包含哪些資訊</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>併入 D2 比對條件(兩者實質相同)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>無付款明細時如何辨識</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>短付/溢付處理及追蹤</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>與 C11 合併為「如何追蹤」;刪除處理方式清單(D5 已涵蓋)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>C. 客戶付款及銀行入帳</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>已匯款未入帳/付款取消的列管及頻率</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>併入 C8;刪除追蹤頻率</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>核對及銷帳負責單位</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>比對條件</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>加入付款明細內容(來自 C8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>比對及銷帳使用系統、自動化程度</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>只保留自動化程度;刪除系統清單</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>一對一/一對多/多對一/部分付款支援</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>4 個子題合為 1 題多選</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>無法辨識/預收款處理及追蹤</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>與 D6 合併為「例外款項如何處理」;刪除追蹤方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>短付/溢付/折讓/減免/其他扣款分類處理</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>5 類款項併入 D5 一題多選</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>核對及銷帳時效、是否有規定時限</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>只保留時效;刪除「是否有規定時限」</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>銷帳日期以何時點為準</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>無變動(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>銷帳後 Outstanding / 放貨 / LFC 是否同步</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>3 個子題合為 1 題</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>銷帳錯誤如何調整及留存紀錄</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>與 D11、D15 合併</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>跨 B/L、跨帳單、跨客戶沖帳</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>併入 D9</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>退款情況、申請單位、核准</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>只保留核准層級;刪除退款情況與申請單位(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>退款前是否先調整原收款及銷帳紀錄</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>退款時效、方式、幣別、帳戶確認</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>D. 核對、銷帳及退款</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>退款是否可追溯至原始紀錄</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>併入 D9 的「並追溯」</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Outstanding Report 來源、頻率、時點</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>3 項縮為「如何產生」;刪除來源系統</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Aging 計算基準及逾期認定</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>只保留計算基準;刪除逾期認定方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>催收頻率及聯繫方式</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>頻率與方式合為一題單選</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>催收紀錄放置系統及內容</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>只保留「放在哪裡」;刪除記錄內容清單</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>爭議款項常見原因</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>是否建立標準原因類型、時限、責任單位</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>與 E7、E8 合併(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>爭議由哪些單位澄清、如何追蹤</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>併入 E6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>E8</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>超過時限的提醒機制</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>併入 E6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>多單位共同管理時如何避免重複/漏催</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>已收款未銷帳是否仍列 Outstanding</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>無變動(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>未收帳款狀態更新頻率及方式</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>併入 E1「如何產生及更新」</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>E. 催收、爭議、高風險客戶</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>高風險客戶名單(條件、核准、註記、限制)</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>E8</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>5 項縮為 1 題:管理方式;刪除列入條件、核准層級、限制內容</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>放貨/放單前確認條件</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Cash/Credit/Central Billing/Non-hold 放行條件</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>4 類客戶縮為 1 題「是否有不同規定」(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Web / Telex / 一般放單的執行單位及系統</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>解除 Hold 的階段及是否自動</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>只保留階段;刪除自動/人工(已併入 D8 同步更新)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>授信客戶額度及逾期檢核方式</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>與 F6 合併</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>信用額度定期檢視(頻率、依據、單位、續核)</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>只保留「是否定期檢視」;刪除依據、負責單位、續核流程</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>緊急放貨/Non-Hold 判斷、核准、記錄</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>與 F9 合併(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款的放貨確認</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>併入 G4</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>F. 放貨 / 放單</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>未銷帳/部分付款/短付時是否可放貨及核准</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>併入 F5</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款發生情況、取得時點及單位</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>只保留發生情況;刪除取得時點與取得單位</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>確認付款人、實際客戶及 B/L、Invoice</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>每月筆數及主要付款地</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>只保留每月筆數區間;刪除付款地(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款涉及的幣別、匯率、銀行帳戶</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>無法確認付款人時如何暫列及追蹤</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>與 G6、F8 合併</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>資訊確認前收款對銷帳/放貨的影響</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>併入 G4</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>G7</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>C/A 通知時點及影響</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款退款情況、申請、核准</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>刪除;核准層級可參考 D10</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>G9</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款退款追溯</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>刪除;追溯性已於 D9 涵蓋</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>G. 第三地付款</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>第三地付款溢付處理</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>併入 D5 例外款項處理</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>LFC 資料產生系統</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>LFC 收入項目及 Non-Manifest/Local Charge 費用項目</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>只保留收入項目類別;刪除費用項目清單(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>LFC 產製/檢核/核准/送檔單位</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>LFC 報收頻率、送檔日期、Cut-off</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>只保留報收頻率;刪除送檔日期與 Cut-off(FRMD 分頁已有報收頻率,可預填)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>LFC 認列依據時點</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>無變動</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>銷帳後多久報收 LFC</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>LFC 可追溯的資料</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>與 H8 合併為「可追溯並核對」</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>LFC 與前端核對及差異處理</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>併入 H5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>H9</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>匯款頻率、日期、Cut-off、換匯時點</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>刪除;FRMD 分頁已有匯款頻率,可預填</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>匯款負責單位、平台、核准流程</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>簡化</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>只保留核准流程;刪除負責單位與平台(列為可選題)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>匯款金額與 LFC 金額差異處理</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>匯款前扣除項目及 LFC 呈現</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>刪除;FRMD 分頁已有手續費資料</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>H13</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>已報收未匯款/已收款未報收的列管</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>刪除,建議於訪談補問</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
           <t>H14</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>各環節幣別是否一致</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>FRMD 分頁已有報收及匯款幣別,可預填</t>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>各環節幣別是否一致及處理</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>刪除</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>刪除;FRMD 分頁已有報收及匯款幣別,可預填</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>H15</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>幣別間使用的匯率</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>保留</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>選項採原題舉例</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>H16</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>不同匯率的差異處理</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>與 H17 合併</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>H17</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>H. LFC 報收及匯款</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>匯兌盈損認列、調整、回報</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>合併</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>併入 H8</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3899,7 +6758,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>合計</t>
         </is>

</xml_diff>